<commit_message>
Show 2023 middle-1 class growth with students labeled A–D and add table/chart slides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bh4sYU41PMoBKwVo8YRab
</commit_message>
<xml_diff>
--- a/output/isabel-cohorts/김건희반_총점_성장.xlsx
+++ b/output/isabel-cohorts/김건희반_총점_성장.xlsx
@@ -134,41 +134,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">수능</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">으</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로 어려워지는데도</t>
+      <t xml:space="preserve">수능 순서로 어려워지는데도</t>
     </r>
     <r>
       <rPr>
@@ -4636,11 +4602,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="57142609"/>
-        <c:axId val="24612484"/>
+        <c:axId val="31546097"/>
+        <c:axId val="25358707"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57142609"/>
+        <c:axId val="31546097"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4672,7 +4638,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24612484"/>
+        <c:crossAx val="25358707"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4680,7 +4646,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24612484"/>
+        <c:axId val="25358707"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -4724,7 +4690,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57142609"/>
+        <c:crossAx val="31546097"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5182,11 +5148,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="61799606"/>
-        <c:axId val="17684708"/>
+        <c:axId val="28417238"/>
+        <c:axId val="87970045"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61799606"/>
+        <c:axId val="28417238"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5218,7 +5184,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17684708"/>
+        <c:crossAx val="87970045"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5226,7 +5192,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17684708"/>
+        <c:axId val="87970045"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -5270,7 +5236,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61799606"/>
+        <c:crossAx val="28417238"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6014,11 +5980,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="30175411"/>
-        <c:axId val="69611161"/>
+        <c:axId val="76637809"/>
+        <c:axId val="59517011"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="30175411"/>
+        <c:axId val="76637809"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6050,7 +6016,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69611161"/>
+        <c:crossAx val="59517011"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6058,7 +6024,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69611161"/>
+        <c:axId val="59517011"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -6136,7 +6102,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30175411"/>
+        <c:crossAx val="76637809"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -6436,11 +6402,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="14442490"/>
-        <c:axId val="12384516"/>
+        <c:axId val="65140394"/>
+        <c:axId val="70178894"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14442490"/>
+        <c:axId val="65140394"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6472,7 +6438,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12384516"/>
+        <c:crossAx val="70178894"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6480,7 +6446,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12384516"/>
+        <c:axId val="70178894"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -6524,7 +6490,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14442490"/>
+        <c:crossAx val="65140394"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7163,11 +7129,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="79847309"/>
-        <c:axId val="57595208"/>
+        <c:axId val="38612303"/>
+        <c:axId val="10835486"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="79847309"/>
+        <c:axId val="38612303"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7199,7 +7165,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57595208"/>
+        <c:crossAx val="10835486"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7207,7 +7173,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57595208"/>
+        <c:axId val="10835486"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -7285,7 +7251,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79847309"/>
+        <c:crossAx val="38612303"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -7585,11 +7551,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="12055881"/>
-        <c:axId val="49015053"/>
+        <c:axId val="3301329"/>
+        <c:axId val="27132951"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="12055881"/>
+        <c:axId val="3301329"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7621,7 +7587,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49015053"/>
+        <c:crossAx val="27132951"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7629,7 +7595,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="49015053"/>
+        <c:axId val="27132951"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -7673,7 +7639,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12055881"/>
+        <c:crossAx val="3301329"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8239,11 +8205,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="63904288"/>
-        <c:axId val="3648430"/>
+        <c:axId val="61110580"/>
+        <c:axId val="59875593"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="63904288"/>
+        <c:axId val="61110580"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8275,7 +8241,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3648430"/>
+        <c:crossAx val="59875593"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8283,7 +8249,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3648430"/>
+        <c:axId val="59875593"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -8361,7 +8327,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63904288"/>
+        <c:crossAx val="61110580"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -8661,11 +8627,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="57453565"/>
-        <c:axId val="43276135"/>
+        <c:axId val="26157242"/>
+        <c:axId val="76689488"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57453565"/>
+        <c:axId val="26157242"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8697,7 +8663,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43276135"/>
+        <c:crossAx val="76689488"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8705,7 +8671,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43276135"/>
+        <c:axId val="76689488"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -8749,7 +8715,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57453565"/>
+        <c:crossAx val="26157242"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>